<commit_message>
edge device benchmark eklendi
</commit_message>
<xml_diff>
--- a/results/benchmark_v3.xlsx
+++ b/results/benchmark_v3.xlsx
@@ -10,7 +10,7 @@
     <sheet r:id="rId1" sheetId="1" name="Summary"/>
     <sheet r:id="rId2" sheetId="2" name="Per-class Accuracy"/>
     <sheet r:id="rId3" sheetId="3" name="Speed Details"/>
-    <sheet r:id="rId4" sheetId="4" name="Memory &amp;amp; Size"/>
+    <sheet r:id="rId4" sheetId="4" name="Memory &amp;amp;amp;amp; Size"/>
   </sheets>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -199,7 +199,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>

</xml_diff>